<commit_message>
Sampling as in the paper: learned variance and colour guidance in the notebook and README; Traffic Signs colour statistics
</commit_message>
<xml_diff>
--- a/evaluation/sheets/Step14_Cityscapes_200k_metrics.xlsx
+++ b/evaluation/sheets/Step14_Cityscapes_200k_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL40"/>
+  <dimension ref="A1:AL43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5486,6 +5486,384 @@
         <v>42</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_wideband35_ema200000_n3000_r500_colsample_anc500_cfg15</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>730.44003</v>
+      </c>
+      <c r="C41" t="n">
+        <v>692.96919</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3.69618</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.07142</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.06133</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.09767000000000001</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.15467</v>
+      </c>
+      <c r="J41" t="n">
+        <v>97.7</v>
+      </c>
+      <c r="K41" t="n">
+        <v>8.500500000000001</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-4.23421</v>
+      </c>
+      <c r="M41" t="n">
+        <v>79.69741</v>
+      </c>
+      <c r="N41" t="n">
+        <v>37.33333</v>
+      </c>
+      <c r="O41" t="n">
+        <v>45.65184</v>
+      </c>
+      <c r="P41" t="n">
+        <v>41.62681</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0.03664</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0.00112</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0.51367</v>
+      </c>
+      <c r="T41" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0.3268</v>
+      </c>
+      <c r="V41" t="n">
+        <v>0.514</v>
+      </c>
+      <c r="W41" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X41" t="n">
+        <v>72.87126922607422</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>5.093384265899658</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>46.92330169677734</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>40.17580795288086</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>652.3410949707031</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>10.402</v>
+      </c>
+      <c r="AF41" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH41" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AI41" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK41" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_wideband35_ema200000_n3000_r500_colsample_anc500_cfg20</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>798.02308</v>
+      </c>
+      <c r="C42" t="n">
+        <v>760.18295</v>
+      </c>
+      <c r="D42" t="n">
+        <v>4.10448</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.07681</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.26867</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.07872999999999999</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.11633</v>
+      </c>
+      <c r="J42" t="n">
+        <v>97.63333</v>
+      </c>
+      <c r="K42" t="n">
+        <v>10.44342</v>
+      </c>
+      <c r="L42" t="n">
+        <v>-3.78707</v>
+      </c>
+      <c r="M42" t="n">
+        <v>78.64878</v>
+      </c>
+      <c r="N42" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="O42" t="n">
+        <v>52.9631</v>
+      </c>
+      <c r="P42" t="n">
+        <v>48.73697</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.04672</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0.00142</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0.24333</v>
+      </c>
+      <c r="V42" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="W42" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X42" t="n">
+        <v>72.97183227539062</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>5.015986919403076</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>48.43784713745117</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>44.94611358642578</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>1001.813690185547</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>1.233333333333333</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>10.338</v>
+      </c>
+      <c r="AF42" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG42" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI42" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ42" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK42" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_wideband35_ema200000_n3000_r500_colsample_anc500_nocfg</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>784.04614</v>
+      </c>
+      <c r="C43" t="n">
+        <v>743.74839</v>
+      </c>
+      <c r="D43" t="n">
+        <v>3.84001</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.07088</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.31533</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.04967</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.09653</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.13433</v>
+      </c>
+      <c r="J43" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="K43" t="n">
+        <v>8.707689999999999</v>
+      </c>
+      <c r="L43" t="n">
+        <v>-1.86253</v>
+      </c>
+      <c r="M43" t="n">
+        <v>81.34638</v>
+      </c>
+      <c r="N43" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="O43" t="n">
+        <v>44.50841</v>
+      </c>
+      <c r="P43" t="n">
+        <v>40.29457</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0.03413</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0.00107</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0.54967</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0.30267</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0.40747</v>
+      </c>
+      <c r="V43" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="W43" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X43" t="n">
+        <v>72.85115814208984</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>5.112388134002686</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>45.14550018310547</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>35.7253532409668</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>363.9930114746094</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>500</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="AF43" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG43" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI43" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ43" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK43" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL43" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Evaluation record: Cityscapes sheets with the box-gradient rows, its bootstrap files and cell, and the table builder behind the current tables
</commit_message>
<xml_diff>
--- a/evaluation/sheets/Step14_Cityscapes_200k_metrics.xlsx
+++ b/evaluation/sheets/Step14_Cityscapes_200k_metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL43"/>
+  <dimension ref="A1:AL46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5864,6 +5864,384 @@
       </c>
       <c r="AL43" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_advbox_ema200000_n3000_r500_colsample_anc500_cfg15</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>560.83653</v>
+      </c>
+      <c r="C44" t="n">
+        <v>520.46914</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2.57889</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.07006</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.25167</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.32627</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.35533</v>
+      </c>
+      <c r="J44" t="n">
+        <v>92</v>
+      </c>
+      <c r="K44" t="n">
+        <v>3.72949</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-10.81805</v>
+      </c>
+      <c r="M44" t="n">
+        <v>82.01862</v>
+      </c>
+      <c r="N44" t="n">
+        <v>39.93333</v>
+      </c>
+      <c r="O44" t="n">
+        <v>22.11654</v>
+      </c>
+      <c r="P44" t="n">
+        <v>18.56761</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.00993</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0.00058</v>
+      </c>
+      <c r="S44" t="n">
+        <v>0.8756699999999999</v>
+      </c>
+      <c r="T44" t="n">
+        <v>0.44433</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.59233</v>
+      </c>
+      <c r="V44" t="n">
+        <v>0.93167</v>
+      </c>
+      <c r="W44" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X44" t="n">
+        <v>72.88507080078125</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>5.121173858642578</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>45.92118835449219</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>35.18685150146484</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>125.002269744873</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>10.35</v>
+      </c>
+      <c r="AF44" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG44" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH44" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AI44" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ44" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK44" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_advbox_ema200000_n3000_r500_colsample_anc500_cfg20</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>541.39807</v>
+      </c>
+      <c r="C45" t="n">
+        <v>500.61745</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2.48565</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.06984</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.27567</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.3412</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="J45" t="n">
+        <v>92.83334000000001</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.94101</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-6.30211</v>
+      </c>
+      <c r="M45" t="n">
+        <v>83.56440000000001</v>
+      </c>
+      <c r="N45" t="n">
+        <v>38.66667</v>
+      </c>
+      <c r="O45" t="n">
+        <v>22.30283</v>
+      </c>
+      <c r="P45" t="n">
+        <v>18.91932</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.01088</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0.00074</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0.873</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.453</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.5266</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0.93267</v>
+      </c>
+      <c r="W45" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X45" t="n">
+        <v>72.95896911621094</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>5.067681312561035</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>48.40306091308594</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>40.06074905395508</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>183.2542877197266</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>10.344</v>
+      </c>
+      <c r="AF45" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG45" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH45" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI45" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ45" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK45" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>cityscapes_fdgan_advbox_ema200000_n3000_r500_colsample_anc500_nocfg</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>746.18272</v>
+      </c>
+      <c r="C46" t="n">
+        <v>709.82284</v>
+      </c>
+      <c r="D46" t="n">
+        <v>3.53824</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.07473</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.49833</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.17967</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.21787</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.26133</v>
+      </c>
+      <c r="J46" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>4.75636</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-14.55036</v>
+      </c>
+      <c r="M46" t="n">
+        <v>79.45129</v>
+      </c>
+      <c r="N46" t="n">
+        <v>39.26667</v>
+      </c>
+      <c r="O46" t="n">
+        <v>30.59326</v>
+      </c>
+      <c r="P46" t="n">
+        <v>27.00502</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.01833</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0.00076</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0.81033</v>
+      </c>
+      <c r="T46" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="U46" t="n">
+        <v>1.25053</v>
+      </c>
+      <c r="V46" t="n">
+        <v>0.84967</v>
+      </c>
+      <c r="W46" t="n">
+        <v>3000</v>
+      </c>
+      <c r="X46" t="n">
+        <v>72.86284637451172</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>5.142828941345215</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>44.23048782348633</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>31.4572811126709</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>85.46933746337891</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>500</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>5.182</v>
+      </c>
+      <c r="AF46" t="inlineStr">
+        <is>
+          <t>NVIDIA A100-SXM4-80GB</t>
+        </is>
+      </c>
+      <c r="AG46" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="AH46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI46" t="inlineStr">
+        <is>
+          <t>predict</t>
+        </is>
+      </c>
+      <c r="AJ46" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="AK46" t="inlineStr">
+        <is>
+          <t>learned</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>